<commit_message>
Mise à jour page Robinetterie
</commit_message>
<xml_diff>
--- a/prix/prix.xlsx
+++ b/prix/prix.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\robinetterie\prix\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C9572EE1-A484-42E3-BBAB-3F376FFEE3E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA670DF4-9488-4F3C-A5AA-B616600FAE31}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{6E95DC93-531D-460D-9A06-44397A8920D7}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="366" uniqueCount="272">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="409" uniqueCount="315">
   <si>
     <t>path</t>
   </si>
@@ -852,6 +852,135 @@
   </si>
   <si>
     <t>79161</t>
+  </si>
+  <si>
+    <t>schutte/24556.png</t>
+  </si>
+  <si>
+    <t>schutte/60170.png</t>
+  </si>
+  <si>
+    <t>schutte/60046.png</t>
+  </si>
+  <si>
+    <t>schutte/60531.png</t>
+  </si>
+  <si>
+    <t>schutte/60690.png</t>
+  </si>
+  <si>
+    <t>schutte/60096.png</t>
+  </si>
+  <si>
+    <t>schutte/60090.png</t>
+  </si>
+  <si>
+    <t>schutte/77440.png</t>
+  </si>
+  <si>
+    <t>schutte/77430.png</t>
+  </si>
+  <si>
+    <t>schutte/44406.png</t>
+  </si>
+  <si>
+    <t>schutte/44306.png</t>
+  </si>
+  <si>
+    <t>schutte/52445.png</t>
+  </si>
+  <si>
+    <t>schutte/33180.png</t>
+  </si>
+  <si>
+    <t>schutte/33186.png</t>
+  </si>
+  <si>
+    <t>schutte/54250.png</t>
+  </si>
+  <si>
+    <t>schutte/33190.png</t>
+  </si>
+  <si>
+    <t>schutte/33196.png</t>
+  </si>
+  <si>
+    <t>schutte/33100.png</t>
+  </si>
+  <si>
+    <t>schutte/33106.png</t>
+  </si>
+  <si>
+    <t>schutte/33120.png</t>
+  </si>
+  <si>
+    <t>schutte/33126.png</t>
+  </si>
+  <si>
+    <t>schutte/33110.png</t>
+  </si>
+  <si>
+    <t>schutte/33116.png</t>
+  </si>
+  <si>
+    <t>schutte/77410.png</t>
+  </si>
+  <si>
+    <t>schutte/44106.png</t>
+  </si>
+  <si>
+    <t>schutte/32210.png</t>
+  </si>
+  <si>
+    <t>schutte/46951.png</t>
+  </si>
+  <si>
+    <t>schutte/37955.png</t>
+  </si>
+  <si>
+    <t>schutte/37965.png</t>
+  </si>
+  <si>
+    <t>schutte/79116.png</t>
+  </si>
+  <si>
+    <t>schutte/79126.png</t>
+  </si>
+  <si>
+    <t>schutte/79760.png</t>
+  </si>
+  <si>
+    <t>schutte/79770.png</t>
+  </si>
+  <si>
+    <t>schutte/79142.png</t>
+  </si>
+  <si>
+    <t>schutte/79147.png</t>
+  </si>
+  <si>
+    <t>schutte/77266.png</t>
+  </si>
+  <si>
+    <t>schutte/35676.png</t>
+  </si>
+  <si>
+    <t>schutte/79616.png</t>
+  </si>
+  <si>
+    <t>schutte/79966.png</t>
+  </si>
+  <si>
+    <t>schutte/79586.png</t>
+  </si>
+  <si>
+    <t>schutte/79162.png</t>
+  </si>
+  <si>
+    <t>schutte/79166.png</t>
+  </si>
+  <si>
+    <t>schutte/79161.png</t>
   </si>
 </sst>
 </file>
@@ -2462,7 +2591,9 @@
       <c r="F52" s="76"/>
     </row>
     <row r="53" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A53" s="5"/>
+      <c r="A53" s="5" t="s">
+        <v>273</v>
+      </c>
       <c r="B53" s="79" t="s">
         <v>188</v>
       </c>
@@ -2486,6 +2617,9 @@
       </c>
     </row>
     <row r="54" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A54" s="4" t="s">
+        <v>274</v>
+      </c>
       <c r="B54" s="79" t="s">
         <v>189</v>
       </c>
@@ -2509,6 +2643,9 @@
       </c>
     </row>
     <row r="55" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A55" s="4" t="s">
+        <v>275</v>
+      </c>
       <c r="B55" s="79" t="s">
         <v>190</v>
       </c>
@@ -2532,6 +2669,9 @@
       </c>
     </row>
     <row r="56" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A56" s="4" t="s">
+        <v>276</v>
+      </c>
       <c r="B56" s="79" t="s">
         <v>191</v>
       </c>
@@ -2555,7 +2695,9 @@
       </c>
     </row>
     <row r="57" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A57" s="5"/>
+      <c r="A57" s="5" t="s">
+        <v>277</v>
+      </c>
       <c r="B57" s="79" t="s">
         <v>192</v>
       </c>
@@ -2579,7 +2721,9 @@
       </c>
     </row>
     <row r="58" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A58" s="5"/>
+      <c r="A58" s="5" t="s">
+        <v>278</v>
+      </c>
       <c r="B58" s="79" t="s">
         <v>193</v>
       </c>
@@ -2603,7 +2747,9 @@
       </c>
     </row>
     <row r="59" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A59" s="5"/>
+      <c r="A59" s="5" t="s">
+        <v>279</v>
+      </c>
       <c r="B59" s="79" t="s">
         <v>194</v>
       </c>
@@ -2627,7 +2773,9 @@
       </c>
     </row>
     <row r="60" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A60" s="5"/>
+      <c r="A60" s="5" t="s">
+        <v>280</v>
+      </c>
       <c r="B60" s="79" t="s">
         <v>195</v>
       </c>
@@ -2652,7 +2800,9 @@
       </c>
     </row>
     <row r="61" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A61" s="5"/>
+      <c r="A61" s="5" t="s">
+        <v>281</v>
+      </c>
       <c r="B61" s="79" t="s">
         <v>196</v>
       </c>
@@ -2677,7 +2827,9 @@
       </c>
     </row>
     <row r="62" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A62" s="5"/>
+      <c r="A62" s="5" t="s">
+        <v>282</v>
+      </c>
       <c r="B62" s="79" t="s">
         <v>197</v>
       </c>
@@ -2702,7 +2854,9 @@
       </c>
     </row>
     <row r="63" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A63" s="5"/>
+      <c r="A63" s="5" t="s">
+        <v>283</v>
+      </c>
       <c r="B63" s="79" t="s">
         <v>198</v>
       </c>
@@ -2726,7 +2880,9 @@
       </c>
     </row>
     <row r="64" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A64" s="5"/>
+      <c r="A64" s="5" t="s">
+        <v>284</v>
+      </c>
       <c r="B64" s="79" t="s">
         <v>199</v>
       </c>
@@ -2750,7 +2906,9 @@
       </c>
     </row>
     <row r="65" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A65" s="5"/>
+      <c r="A65" s="5" t="s">
+        <v>285</v>
+      </c>
       <c r="B65" s="79" t="s">
         <v>200</v>
       </c>
@@ -2774,7 +2932,9 @@
       </c>
     </row>
     <row r="66" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A66" s="5"/>
+      <c r="A66" s="5" t="s">
+        <v>286</v>
+      </c>
       <c r="B66" s="79" t="s">
         <v>201</v>
       </c>
@@ -2798,7 +2958,9 @@
       </c>
     </row>
     <row r="67" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A67" s="5"/>
+      <c r="A67" s="5" t="s">
+        <v>287</v>
+      </c>
       <c r="B67" s="79" t="s">
         <v>202</v>
       </c>
@@ -2822,7 +2984,9 @@
       </c>
     </row>
     <row r="68" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A68" s="5"/>
+      <c r="A68" s="5" t="s">
+        <v>288</v>
+      </c>
       <c r="B68" s="79" t="s">
         <v>203</v>
       </c>
@@ -2846,7 +3010,9 @@
       </c>
     </row>
     <row r="69" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A69" s="5"/>
+      <c r="A69" s="5" t="s">
+        <v>289</v>
+      </c>
       <c r="B69" s="79" t="s">
         <v>204</v>
       </c>
@@ -2870,7 +3036,9 @@
       </c>
     </row>
     <row r="70" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A70" s="5"/>
+      <c r="A70" s="5" t="s">
+        <v>290</v>
+      </c>
       <c r="B70" s="79" t="s">
         <v>205</v>
       </c>
@@ -2894,7 +3062,9 @@
       </c>
     </row>
     <row r="71" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A71" s="5"/>
+      <c r="A71" s="5" t="s">
+        <v>291</v>
+      </c>
       <c r="B71" s="79" t="s">
         <v>204</v>
       </c>
@@ -2918,7 +3088,9 @@
       </c>
     </row>
     <row r="72" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A72" s="5"/>
+      <c r="A72" s="5" t="s">
+        <v>292</v>
+      </c>
       <c r="B72" s="79" t="s">
         <v>205</v>
       </c>
@@ -2942,7 +3114,9 @@
       </c>
     </row>
     <row r="73" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A73" s="5"/>
+      <c r="A73" s="5" t="s">
+        <v>293</v>
+      </c>
       <c r="B73" s="79" t="s">
         <v>206</v>
       </c>
@@ -2966,7 +3140,9 @@
       </c>
     </row>
     <row r="74" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A74" s="5"/>
+      <c r="A74" s="5" t="s">
+        <v>294</v>
+      </c>
       <c r="B74" s="79" t="s">
         <v>207</v>
       </c>
@@ -2990,7 +3166,9 @@
       </c>
     </row>
     <row r="75" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A75" s="5"/>
+      <c r="A75" s="5" t="s">
+        <v>295</v>
+      </c>
       <c r="B75" s="79" t="s">
         <v>208</v>
       </c>
@@ -3014,7 +3192,9 @@
       </c>
     </row>
     <row r="76" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A76" s="5"/>
+      <c r="A76" s="5" t="s">
+        <v>296</v>
+      </c>
       <c r="B76" s="79" t="s">
         <v>209</v>
       </c>
@@ -3038,7 +3218,9 @@
       </c>
     </row>
     <row r="77" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A77" s="5"/>
+      <c r="A77" s="5" t="s">
+        <v>297</v>
+      </c>
       <c r="B77" s="79" t="s">
         <v>210</v>
       </c>
@@ -3062,7 +3244,9 @@
       </c>
     </row>
     <row r="78" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A78" s="5"/>
+      <c r="A78" s="5" t="s">
+        <v>298</v>
+      </c>
       <c r="B78" s="79" t="s">
         <v>211</v>
       </c>
@@ -3086,7 +3270,9 @@
       </c>
     </row>
     <row r="79" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A79" s="5"/>
+      <c r="A79" s="5" t="s">
+        <v>299</v>
+      </c>
       <c r="B79" s="79" t="s">
         <v>212</v>
       </c>
@@ -3110,7 +3296,9 @@
       </c>
     </row>
     <row r="80" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A80" s="5"/>
+      <c r="A80" s="5" t="s">
+        <v>300</v>
+      </c>
       <c r="B80" s="79" t="s">
         <v>213</v>
       </c>
@@ -3134,7 +3322,9 @@
       </c>
     </row>
     <row r="81" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A81" s="5"/>
+      <c r="A81" s="5" t="s">
+        <v>301</v>
+      </c>
       <c r="B81" s="79" t="s">
         <v>214</v>
       </c>
@@ -3158,7 +3348,9 @@
       </c>
     </row>
     <row r="82" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A82" s="5"/>
+      <c r="A82" s="5" t="s">
+        <v>302</v>
+      </c>
       <c r="B82" s="79" t="s">
         <v>215</v>
       </c>
@@ -3182,7 +3374,9 @@
       </c>
     </row>
     <row r="83" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A83" s="5"/>
+      <c r="A83" s="5" t="s">
+        <v>303</v>
+      </c>
       <c r="B83" s="79" t="s">
         <v>216</v>
       </c>
@@ -3207,7 +3401,9 @@
       </c>
     </row>
     <row r="84" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A84" s="5"/>
+      <c r="A84" s="5" t="s">
+        <v>304</v>
+      </c>
       <c r="B84" s="79" t="s">
         <v>217</v>
       </c>
@@ -3232,7 +3428,9 @@
       </c>
     </row>
     <row r="85" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A85" s="5"/>
+      <c r="A85" s="5" t="s">
+        <v>305</v>
+      </c>
       <c r="B85" s="79" t="s">
         <v>218</v>
       </c>
@@ -3257,7 +3455,9 @@
       </c>
     </row>
     <row r="86" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A86" s="5"/>
+      <c r="A86" s="5" t="s">
+        <v>306</v>
+      </c>
       <c r="B86" s="79" t="s">
         <v>219</v>
       </c>
@@ -3282,7 +3482,9 @@
       </c>
     </row>
     <row r="87" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A87" s="5"/>
+      <c r="A87" s="5" t="s">
+        <v>307</v>
+      </c>
       <c r="B87" s="79" t="s">
         <v>220</v>
       </c>
@@ -3307,7 +3509,9 @@
       </c>
     </row>
     <row r="88" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A88" s="5"/>
+      <c r="A88" s="5" t="s">
+        <v>308</v>
+      </c>
       <c r="B88" s="79" t="s">
         <v>221</v>
       </c>
@@ -3332,7 +3536,9 @@
       </c>
     </row>
     <row r="89" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A89" s="5"/>
+      <c r="A89" s="5" t="s">
+        <v>309</v>
+      </c>
       <c r="B89" s="79" t="s">
         <v>222</v>
       </c>
@@ -3357,7 +3563,9 @@
       </c>
     </row>
     <row r="90" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A90" s="5"/>
+      <c r="A90" s="5" t="s">
+        <v>272</v>
+      </c>
       <c r="B90" s="79" t="s">
         <v>223</v>
       </c>
@@ -3382,7 +3590,9 @@
       </c>
     </row>
     <row r="91" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A91" s="5"/>
+      <c r="A91" s="5" t="s">
+        <v>310</v>
+      </c>
       <c r="B91" s="79" t="s">
         <v>224</v>
       </c>
@@ -3407,7 +3617,9 @@
       </c>
     </row>
     <row r="92" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A92" s="5"/>
+      <c r="A92" s="5" t="s">
+        <v>311</v>
+      </c>
       <c r="B92" s="79" t="s">
         <v>225</v>
       </c>
@@ -3432,7 +3644,9 @@
       </c>
     </row>
     <row r="93" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A93" s="5"/>
+      <c r="A93" s="5" t="s">
+        <v>312</v>
+      </c>
       <c r="B93" s="79" t="s">
         <v>226</v>
       </c>
@@ -3457,7 +3671,9 @@
       </c>
     </row>
     <row r="94" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A94" s="5"/>
+      <c r="A94" s="5" t="s">
+        <v>313</v>
+      </c>
       <c r="B94" s="79" t="s">
         <v>227</v>
       </c>
@@ -3482,7 +3698,9 @@
       </c>
     </row>
     <row r="95" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A95" s="5"/>
+      <c r="A95" s="5" t="s">
+        <v>314</v>
+      </c>
       <c r="B95" s="79" t="s">
         <v>228</v>
       </c>

</xml_diff>